<commit_message>
Add compare-all-sheets, mapping files with formulas and plain-English logic
- Compare every sheet with the same name in both files
- Mapping file maps File 1 columns/formulas to File 2 columns/formulas,
  with keys and per-row tolerance; 'Make template' builds a starter
- Safe vectorised Excel-style formula engine
- Plain-English logic converted to formulas via Claude (claude-opus-5-5)
- 38 new tests (69 total), test data and test plan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/B2B_file1.xlsx
+++ b/test_data/B2B_file1.xlsx
@@ -5759,16 +5759,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL2">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM2">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN2">
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP2">
         <v>0</v>
@@ -6530,16 +6530,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL5">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM5">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -7301,16 +7301,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL8">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM8">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN8">
         <v>0</v>
       </c>
       <c r="AO8">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP8">
         <v>0</v>
@@ -8072,16 +8072,16 @@
         <v>508.47</v>
       </c>
       <c r="AL11">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM11">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN11">
         <v>0</v>
       </c>
       <c r="AO11">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP11">
         <v>0</v>
@@ -8855,16 +8855,16 @@
         <v>1652.54</v>
       </c>
       <c r="AL14">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AM14">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AN14">
         <v>0</v>
       </c>
       <c r="AO14">
-        <v>297.46</v>
+        <v>0</v>
       </c>
       <c r="AP14">
         <v>0</v>
@@ -9626,16 +9626,16 @@
         <v>677.97</v>
       </c>
       <c r="AL17">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM17">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN17">
         <v>0</v>
       </c>
       <c r="AO17">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP17">
         <v>0</v>
@@ -10397,16 +10397,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL20">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM20">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN20">
         <v>0</v>
       </c>
       <c r="AO20">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP20">
         <v>0</v>
@@ -11180,16 +11180,16 @@
         <v>677.97</v>
       </c>
       <c r="AL23">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM23">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN23">
         <v>0</v>
       </c>
       <c r="AO23">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP23">
         <v>0</v>
@@ -11951,16 +11951,16 @@
         <v>677.97</v>
       </c>
       <c r="AL26">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM26">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN26">
         <v>0</v>
       </c>
       <c r="AO26">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP26">
         <v>0</v>
@@ -12728,16 +12728,16 @@
         <v>169.49</v>
       </c>
       <c r="AL29">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM29">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN29">
         <v>0</v>
       </c>
       <c r="AO29">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP29">
         <v>0</v>
@@ -13505,16 +13505,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL32">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM32">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN32">
         <v>0</v>
       </c>
       <c r="AO32">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP32">
         <v>0</v>
@@ -14276,16 +14276,16 @@
         <v>508.47</v>
       </c>
       <c r="AL35">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM35">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN35">
         <v>0</v>
       </c>
       <c r="AO35">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP35">
         <v>0</v>
@@ -15053,16 +15053,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL38">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM38">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN38">
         <v>0</v>
       </c>
       <c r="AO38">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP38">
         <v>0</v>
@@ -15830,16 +15830,16 @@
         <v>550.85</v>
       </c>
       <c r="AL41">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM41">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN41">
         <v>0</v>
       </c>
       <c r="AO41">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP41">
         <v>0</v>
@@ -16607,16 +16607,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL44">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM44">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN44">
         <v>0</v>
       </c>
       <c r="AO44">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP44">
         <v>0</v>
@@ -17384,16 +17384,16 @@
         <v>508.47</v>
       </c>
       <c r="AL47">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM47">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN47">
         <v>0</v>
       </c>
       <c r="AO47">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP47">
         <v>0</v>
@@ -18155,16 +18155,16 @@
         <v>423.73</v>
       </c>
       <c r="AL50">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM50">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN50">
         <v>0</v>
       </c>
       <c r="AO50">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP50">
         <v>0</v>
@@ -18932,16 +18932,16 @@
         <v>338.14</v>
       </c>
       <c r="AL53">
-        <v>0</v>
+        <v>30.43</v>
       </c>
       <c r="AM53">
-        <v>0</v>
+        <v>30.43</v>
       </c>
       <c r="AN53">
         <v>0</v>
       </c>
       <c r="AO53">
-        <v>60.86</v>
+        <v>0</v>
       </c>
       <c r="AP53">
         <v>0</v>
@@ -19709,16 +19709,16 @@
         <v>1652.54</v>
       </c>
       <c r="AL56">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AM56">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AN56">
         <v>0</v>
       </c>
       <c r="AO56">
-        <v>297.46</v>
+        <v>0</v>
       </c>
       <c r="AP56">
         <v>0</v>
@@ -20486,16 +20486,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL59">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM59">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN59">
         <v>0</v>
       </c>
       <c r="AO59">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP59">
         <v>0</v>
@@ -21269,16 +21269,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL62">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM62">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN62">
         <v>0</v>
       </c>
       <c r="AO62">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP62">
         <v>0</v>
@@ -22040,16 +22040,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL65">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM65">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN65">
         <v>0</v>
       </c>
       <c r="AO65">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP65">
         <v>0</v>
@@ -22817,16 +22817,16 @@
         <v>169.49</v>
       </c>
       <c r="AL68">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM68">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN68">
         <v>0</v>
       </c>
       <c r="AO68">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP68">
         <v>0</v>
@@ -23594,16 +23594,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL71">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM71">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN71">
         <v>0</v>
       </c>
       <c r="AO71">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP71">
         <v>0</v>
@@ -24365,16 +24365,16 @@
         <v>423.73</v>
       </c>
       <c r="AL74">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM74">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN74">
         <v>0</v>
       </c>
       <c r="AO74">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP74">
         <v>0</v>
@@ -25142,16 +25142,16 @@
         <v>423.73</v>
       </c>
       <c r="AL77">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM77">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN77">
         <v>0</v>
       </c>
       <c r="AO77">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP77">
         <v>0</v>
@@ -25919,16 +25919,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL80">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM80">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN80">
         <v>0</v>
       </c>
       <c r="AO80">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP80">
         <v>0</v>
@@ -26690,16 +26690,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL83">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM83">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN83">
         <v>0</v>
       </c>
       <c r="AO83">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP83">
         <v>0</v>
@@ -27461,16 +27461,16 @@
         <v>550.85</v>
       </c>
       <c r="AL86">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM86">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN86">
         <v>0</v>
       </c>
       <c r="AO86">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP86">
         <v>0</v>
@@ -28232,16 +28232,16 @@
         <v>508.47</v>
       </c>
       <c r="AL89">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM89">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN89">
         <v>0</v>
       </c>
       <c r="AO89">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP89">
         <v>0</v>
@@ -29003,16 +29003,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL92">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM92">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN92">
         <v>0</v>
       </c>
       <c r="AO92">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP92">
         <v>0</v>
@@ -29780,16 +29780,16 @@
         <v>423.73</v>
       </c>
       <c r="AL95">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM95">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN95">
         <v>0</v>
       </c>
       <c r="AO95">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP95">
         <v>0</v>
@@ -30551,16 +30551,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL98">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM98">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN98">
         <v>0</v>
       </c>
       <c r="AO98">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP98">
         <v>0</v>
@@ -31322,16 +31322,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL101">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM101">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN101">
         <v>0</v>
       </c>
       <c r="AO101">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP101">
         <v>0</v>
@@ -32093,16 +32093,16 @@
         <v>677.97</v>
       </c>
       <c r="AL104">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM104">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN104">
         <v>0</v>
       </c>
       <c r="AO104">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP104">
         <v>0</v>
@@ -32870,16 +32870,16 @@
         <v>676.27</v>
       </c>
       <c r="AL107">
-        <v>0</v>
+        <v>60.86</v>
       </c>
       <c r="AM107">
-        <v>0</v>
+        <v>60.87</v>
       </c>
       <c r="AN107">
         <v>0</v>
       </c>
       <c r="AO107">
-        <v>121.73</v>
+        <v>0</v>
       </c>
       <c r="AP107">
         <v>0</v>
@@ -33647,16 +33647,16 @@
         <v>169.49</v>
       </c>
       <c r="AL110">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM110">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN110">
         <v>0</v>
       </c>
       <c r="AO110">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP110">
         <v>0</v>
@@ -34418,16 +34418,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL113">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM113">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN113">
         <v>0</v>
       </c>
       <c r="AO113">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP113">
         <v>0</v>
@@ -35189,16 +35189,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL116">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM116">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN116">
         <v>0</v>
       </c>
       <c r="AO116">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP116">
         <v>0</v>
@@ -35960,16 +35960,16 @@
         <v>677.97</v>
       </c>
       <c r="AL119">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM119">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN119">
         <v>0</v>
       </c>
       <c r="AO119">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP119">
         <v>0</v>
@@ -36737,16 +36737,16 @@
         <v>338.98</v>
       </c>
       <c r="AL122">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AM122">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AN122">
         <v>0</v>
       </c>
       <c r="AO122">
-        <v>61.02</v>
+        <v>0</v>
       </c>
       <c r="AP122">
         <v>0</v>
@@ -37514,16 +37514,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL125">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM125">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN125">
         <v>0</v>
       </c>
       <c r="AO125">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP125">
         <v>0</v>
@@ -38285,16 +38285,16 @@
         <v>1352.54</v>
       </c>
       <c r="AL128">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AM128">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AN128">
         <v>0</v>
       </c>
       <c r="AO128">
-        <v>243.46</v>
+        <v>0</v>
       </c>
       <c r="AP128">
         <v>0</v>
@@ -39056,16 +39056,16 @@
         <v>169.49</v>
       </c>
       <c r="AL131">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM131">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN131">
         <v>0</v>
       </c>
       <c r="AO131">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP131">
         <v>0</v>
@@ -39827,16 +39827,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL134">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM134">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN134">
         <v>0</v>
       </c>
       <c r="AO134">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP134">
         <v>0</v>
@@ -40598,16 +40598,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL137">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM137">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN137">
         <v>0</v>
       </c>
       <c r="AO137">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP137">
         <v>0</v>
@@ -41381,16 +41381,16 @@
         <v>508.47</v>
       </c>
       <c r="AL140">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM140">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN140">
         <v>0</v>
       </c>
       <c r="AO140">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP140">
         <v>0</v>
@@ -42158,16 +42158,16 @@
         <v>676.27</v>
       </c>
       <c r="AL143">
-        <v>0</v>
+        <v>60.86</v>
       </c>
       <c r="AM143">
-        <v>0</v>
+        <v>60.87</v>
       </c>
       <c r="AN143">
         <v>0</v>
       </c>
       <c r="AO143">
-        <v>121.73</v>
+        <v>0</v>
       </c>
       <c r="AP143">
         <v>0</v>
@@ -42929,16 +42929,16 @@
         <v>676.27</v>
       </c>
       <c r="AL146">
-        <v>0</v>
+        <v>60.86</v>
       </c>
       <c r="AM146">
-        <v>0</v>
+        <v>60.87</v>
       </c>
       <c r="AN146">
         <v>0</v>
       </c>
       <c r="AO146">
-        <v>121.73</v>
+        <v>0</v>
       </c>
       <c r="AP146">
         <v>0</v>
@@ -43706,16 +43706,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL149">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM149">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN149">
         <v>0</v>
       </c>
       <c r="AO149">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP149">
         <v>0</v>
@@ -44477,16 +44477,16 @@
         <v>423.73</v>
       </c>
       <c r="AL152">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM152">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN152">
         <v>0</v>
       </c>
       <c r="AO152">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP152">
         <v>0</v>
@@ -45254,16 +45254,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL155">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM155">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN155">
         <v>0</v>
       </c>
       <c r="AO155">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP155">
         <v>0</v>
@@ -46031,16 +46031,16 @@
         <v>169.49</v>
       </c>
       <c r="AL158">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM158">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN158">
         <v>0</v>
       </c>
       <c r="AO158">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP158">
         <v>0</v>
@@ -46802,16 +46802,16 @@
         <v>550.85</v>
       </c>
       <c r="AL161">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM161">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN161">
         <v>0</v>
       </c>
       <c r="AO161">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP161">
         <v>0</v>
@@ -47573,16 +47573,16 @@
         <v>423.73</v>
       </c>
       <c r="AL164">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM164">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN164">
         <v>0</v>
       </c>
       <c r="AO164">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP164">
         <v>0</v>
@@ -48344,16 +48344,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL167">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM167">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN167">
         <v>0</v>
       </c>
       <c r="AO167">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP167">
         <v>0</v>
@@ -49115,16 +49115,16 @@
         <v>423.73</v>
       </c>
       <c r="AL170">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM170">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN170">
         <v>0</v>
       </c>
       <c r="AO170">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP170">
         <v>0</v>
@@ -49892,16 +49892,16 @@
         <v>677.97</v>
       </c>
       <c r="AL173">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM173">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN173">
         <v>0</v>
       </c>
       <c r="AO173">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP173">
         <v>0</v>
@@ -50663,16 +50663,16 @@
         <v>1694.92</v>
       </c>
       <c r="AL176">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AM176">
-        <v>0</v>
+        <v>152.54</v>
       </c>
       <c r="AN176">
         <v>0</v>
       </c>
       <c r="AO176">
-        <v>305.08</v>
+        <v>0</v>
       </c>
       <c r="AP176">
         <v>0</v>
@@ -51434,16 +51434,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL179">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM179">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN179">
         <v>0</v>
       </c>
       <c r="AO179">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP179">
         <v>0</v>
@@ -52217,16 +52217,16 @@
         <v>550.85</v>
       </c>
       <c r="AL182">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM182">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN182">
         <v>0</v>
       </c>
       <c r="AO182">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP182">
         <v>0</v>
@@ -52988,16 +52988,16 @@
         <v>550.85</v>
       </c>
       <c r="AL185">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM185">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN185">
         <v>0</v>
       </c>
       <c r="AO185">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP185">
         <v>0</v>
@@ -53765,16 +53765,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL188">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM188">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN188">
         <v>0</v>
       </c>
       <c r="AO188">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP188">
         <v>0</v>
@@ -54542,16 +54542,16 @@
         <v>676.27</v>
       </c>
       <c r="AL191">
-        <v>0</v>
+        <v>60.86</v>
       </c>
       <c r="AM191">
-        <v>0</v>
+        <v>60.87</v>
       </c>
       <c r="AN191">
         <v>0</v>
       </c>
       <c r="AO191">
-        <v>121.73</v>
+        <v>0</v>
       </c>
       <c r="AP191">
         <v>0</v>
@@ -55319,16 +55319,16 @@
         <v>550.85</v>
       </c>
       <c r="AL194">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM194">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN194">
         <v>0</v>
       </c>
       <c r="AO194">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP194">
         <v>0</v>
@@ -56090,16 +56090,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL197">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM197">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN197">
         <v>0</v>
       </c>
       <c r="AO197">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP197">
         <v>0</v>
@@ -56861,16 +56861,16 @@
         <v>1652.54</v>
       </c>
       <c r="AL200">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AM200">
-        <v>0</v>
+        <v>148.73</v>
       </c>
       <c r="AN200">
         <v>0</v>
       </c>
       <c r="AO200">
-        <v>297.46</v>
+        <v>0</v>
       </c>
       <c r="AP200">
         <v>0</v>
@@ -57632,16 +57632,16 @@
         <v>169.49</v>
       </c>
       <c r="AL203">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM203">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN203">
         <v>0</v>
       </c>
       <c r="AO203">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP203">
         <v>0</v>
@@ -58403,16 +58403,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL206">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM206">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN206">
         <v>0</v>
       </c>
       <c r="AO206">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP206">
         <v>0</v>
@@ -59180,16 +59180,16 @@
         <v>338.98</v>
       </c>
       <c r="AL209">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AM209">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AN209">
         <v>0</v>
       </c>
       <c r="AO209">
-        <v>61.02</v>
+        <v>0</v>
       </c>
       <c r="AP209">
         <v>0</v>
@@ -59957,16 +59957,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL212">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM212">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN212">
         <v>0</v>
       </c>
       <c r="AO212">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP212">
         <v>0</v>
@@ -60728,16 +60728,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL215">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM215">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN215">
         <v>0</v>
       </c>
       <c r="AO215">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP215">
         <v>0</v>
@@ -61505,16 +61505,16 @@
         <v>676.27</v>
       </c>
       <c r="AL218">
-        <v>0</v>
+        <v>60.86</v>
       </c>
       <c r="AM218">
-        <v>0</v>
+        <v>60.87</v>
       </c>
       <c r="AN218">
         <v>0</v>
       </c>
       <c r="AO218">
-        <v>121.73</v>
+        <v>0</v>
       </c>
       <c r="AP218">
         <v>0</v>
@@ -62276,16 +62276,16 @@
         <v>1352.54</v>
       </c>
       <c r="AL221">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AM221">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AN221">
         <v>0</v>
       </c>
       <c r="AO221">
-        <v>243.46</v>
+        <v>0</v>
       </c>
       <c r="AP221">
         <v>0</v>
@@ -63053,16 +63053,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL224">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM224">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN224">
         <v>0</v>
       </c>
       <c r="AO224">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP224">
         <v>0</v>
@@ -63830,16 +63830,16 @@
         <v>847.46</v>
       </c>
       <c r="AL227">
-        <v>0</v>
+        <v>76.27</v>
       </c>
       <c r="AM227">
-        <v>0</v>
+        <v>76.27</v>
       </c>
       <c r="AN227">
         <v>0</v>
       </c>
       <c r="AO227">
-        <v>152.54</v>
+        <v>0</v>
       </c>
       <c r="AP227">
         <v>0</v>
@@ -64607,16 +64607,16 @@
         <v>677.97</v>
       </c>
       <c r="AL230">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM230">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN230">
         <v>0</v>
       </c>
       <c r="AO230">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP230">
         <v>0</v>
@@ -65384,16 +65384,16 @@
         <v>1352.54</v>
       </c>
       <c r="AL233">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AM233">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AN233">
         <v>0</v>
       </c>
       <c r="AO233">
-        <v>243.46</v>
+        <v>0</v>
       </c>
       <c r="AP233">
         <v>0</v>
@@ -66155,16 +66155,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL236">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM236">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN236">
         <v>0</v>
       </c>
       <c r="AO236">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP236">
         <v>0</v>
@@ -66932,16 +66932,16 @@
         <v>550.85</v>
       </c>
       <c r="AL239">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM239">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN239">
         <v>0</v>
       </c>
       <c r="AO239">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP239">
         <v>0</v>
@@ -67703,16 +67703,16 @@
         <v>338.14</v>
       </c>
       <c r="AL242">
-        <v>0</v>
+        <v>30.43</v>
       </c>
       <c r="AM242">
-        <v>0</v>
+        <v>30.43</v>
       </c>
       <c r="AN242">
         <v>0</v>
       </c>
       <c r="AO242">
-        <v>60.86</v>
+        <v>0</v>
       </c>
       <c r="AP242">
         <v>0</v>
@@ -68486,16 +68486,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL245">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM245">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN245">
         <v>0</v>
       </c>
       <c r="AO245">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP245">
         <v>0</v>
@@ -69263,16 +69263,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL248">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM248">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN248">
         <v>0</v>
       </c>
       <c r="AO248">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP248">
         <v>0</v>
@@ -70034,16 +70034,16 @@
         <v>508.47</v>
       </c>
       <c r="AL251">
-        <v>0</v>
+        <v>45.76</v>
       </c>
       <c r="AM251">
-        <v>0</v>
+        <v>45.77</v>
       </c>
       <c r="AN251">
         <v>0</v>
       </c>
       <c r="AO251">
-        <v>91.53</v>
+        <v>0</v>
       </c>
       <c r="AP251">
         <v>0</v>
@@ -70805,16 +70805,16 @@
         <v>1101.69</v>
       </c>
       <c r="AL254">
-        <v>0</v>
+        <v>99.16</v>
       </c>
       <c r="AM254">
-        <v>0</v>
+        <v>99.15000000000001</v>
       </c>
       <c r="AN254">
         <v>0</v>
       </c>
       <c r="AO254">
-        <v>198.31</v>
+        <v>0</v>
       </c>
       <c r="AP254">
         <v>0</v>
@@ -71576,16 +71576,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL257">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM257">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN257">
         <v>0</v>
       </c>
       <c r="AO257">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP257">
         <v>0</v>
@@ -72347,16 +72347,16 @@
         <v>338.98</v>
       </c>
       <c r="AL260">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AM260">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AN260">
         <v>0</v>
       </c>
       <c r="AO260">
-        <v>61.02</v>
+        <v>0</v>
       </c>
       <c r="AP260">
         <v>0</v>
@@ -73130,16 +73130,16 @@
         <v>550.85</v>
       </c>
       <c r="AL263">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM263">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN263">
         <v>0</v>
       </c>
       <c r="AO263">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP263">
         <v>0</v>
@@ -73907,16 +73907,16 @@
         <v>2203.39</v>
       </c>
       <c r="AL266">
-        <v>0</v>
+        <v>198.3</v>
       </c>
       <c r="AM266">
-        <v>0</v>
+        <v>198.31</v>
       </c>
       <c r="AN266">
         <v>0</v>
       </c>
       <c r="AO266">
-        <v>396.61</v>
+        <v>0</v>
       </c>
       <c r="AP266">
         <v>0</v>
@@ -74678,16 +74678,16 @@
         <v>423.73</v>
       </c>
       <c r="AL269">
-        <v>0</v>
+        <v>38.14</v>
       </c>
       <c r="AM269">
-        <v>0</v>
+        <v>38.13</v>
       </c>
       <c r="AN269">
         <v>0</v>
       </c>
       <c r="AO269">
-        <v>76.27</v>
+        <v>0</v>
       </c>
       <c r="AP269">
         <v>0</v>
@@ -75449,16 +75449,16 @@
         <v>550.85</v>
       </c>
       <c r="AL272">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM272">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN272">
         <v>0</v>
       </c>
       <c r="AO272">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP272">
         <v>0</v>
@@ -76232,16 +76232,16 @@
         <v>1352.54</v>
       </c>
       <c r="AL275">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AM275">
-        <v>0</v>
+        <v>121.73</v>
       </c>
       <c r="AN275">
         <v>0</v>
       </c>
       <c r="AO275">
-        <v>243.46</v>
+        <v>0</v>
       </c>
       <c r="AP275">
         <v>0</v>
@@ -77003,16 +77003,16 @@
         <v>847.46</v>
       </c>
       <c r="AL278">
-        <v>0</v>
+        <v>76.27</v>
       </c>
       <c r="AM278">
-        <v>0</v>
+        <v>76.27</v>
       </c>
       <c r="AN278">
         <v>0</v>
       </c>
       <c r="AO278">
-        <v>152.54</v>
+        <v>0</v>
       </c>
       <c r="AP278">
         <v>0</v>
@@ -77774,16 +77774,16 @@
         <v>550.85</v>
       </c>
       <c r="AL281">
-        <v>0</v>
+        <v>49.58</v>
       </c>
       <c r="AM281">
-        <v>0</v>
+        <v>49.57000000000001</v>
       </c>
       <c r="AN281">
         <v>0</v>
       </c>
       <c r="AO281">
-        <v>99.15000000000001</v>
+        <v>0</v>
       </c>
       <c r="AP281">
         <v>0</v>
@@ -78551,16 +78551,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL284">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM284">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN284">
         <v>0</v>
       </c>
       <c r="AO284">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP284">
         <v>0</v>
@@ -79322,16 +79322,16 @@
         <v>338.98</v>
       </c>
       <c r="AL287">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AM287">
-        <v>0</v>
+        <v>30.51</v>
       </c>
       <c r="AN287">
         <v>0</v>
       </c>
       <c r="AO287">
-        <v>61.02</v>
+        <v>0</v>
       </c>
       <c r="AP287">
         <v>0</v>
@@ -80093,16 +80093,16 @@
         <v>1271.19</v>
       </c>
       <c r="AL290">
-        <v>0</v>
+        <v>114.4</v>
       </c>
       <c r="AM290">
-        <v>0</v>
+        <v>114.41</v>
       </c>
       <c r="AN290">
         <v>0</v>
       </c>
       <c r="AO290">
-        <v>228.81</v>
+        <v>0</v>
       </c>
       <c r="AP290">
         <v>0</v>
@@ -80864,16 +80864,16 @@
         <v>677.97</v>
       </c>
       <c r="AL293">
-        <v>0</v>
+        <v>61.02</v>
       </c>
       <c r="AM293">
-        <v>0</v>
+        <v>61.01</v>
       </c>
       <c r="AN293">
         <v>0</v>
       </c>
       <c r="AO293">
-        <v>122.03</v>
+        <v>0</v>
       </c>
       <c r="AP293">
         <v>0</v>
@@ -81641,16 +81641,16 @@
         <v>169.49</v>
       </c>
       <c r="AL296">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="AM296">
-        <v>0</v>
+        <v>15.25</v>
       </c>
       <c r="AN296">
         <v>0</v>
       </c>
       <c r="AO296">
-        <v>30.51</v>
+        <v>0</v>
       </c>
       <c r="AP296">
         <v>0</v>
@@ -82412,16 +82412,16 @@
         <v>1014.41</v>
       </c>
       <c r="AL299">
-        <v>0</v>
+        <v>91.3</v>
       </c>
       <c r="AM299">
-        <v>0</v>
+        <v>91.29000000000001</v>
       </c>
       <c r="AN299">
         <v>0</v>
       </c>
       <c r="AO299">
-        <v>182.59</v>
+        <v>0</v>
       </c>
       <c r="AP299">
         <v>0</v>

</xml_diff>